<commit_message>
Remove every mention of the supplier by name
A retailer should not advertise who it buys from: customers can go direct
and competitors learn the supply chain.

Site copy: "Catalogue IFDC" becomes "Catalogue complet", "Distributeur
autorisé IFDC" becomes "Distributeur autorisé", and the intro and note no
longer say where the photographs come from. Page titles, meta and
og:description follow.

Also scrubbed from places the public repository exposes: identifiers,
class names, data filenames, the fetch script, the README, and the "Source
du prix" column of the review spreadsheet. The harvested data carried the
supplier's product-page URL on all 976 rows for provenance the site never
used — the field is dropped and no longer recorded.

Product codes (IF-, T-, C-) stay: they are the store's own SKUs and appear
on the products themselves.

Zero mentions remain in the built site or in any tracked source file.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/exports/revision-prix.xlsx
+++ b/web/exports/revision-prix.xlsx
@@ -750,7 +750,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I6" s="6" t="n"/>
@@ -795,7 +795,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I7" s="6" t="n"/>
@@ -840,7 +840,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I27" s="6" t="n"/>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I61" s="6" t="n"/>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="H64" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I64" s="6" t="n"/>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="H65" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I65" s="6" t="n"/>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="H68" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I68" s="6" t="n"/>
@@ -2985,7 +2985,7 @@
       </c>
       <c r="H69" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I69" s="6" t="n"/>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="H70" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I70" s="6" t="n"/>
@@ -3504,7 +3504,7 @@
       </c>
       <c r="H84" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I84" s="6" t="n"/>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="H85" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I85" s="6" t="n"/>
@@ -3586,7 +3586,7 @@
       </c>
       <c r="H86" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I86" s="6" t="n"/>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="H87" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I87" s="6" t="n"/>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="H88" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I88" s="6" t="n"/>
@@ -3709,7 +3709,7 @@
       </c>
       <c r="H89" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I89" s="6" t="n"/>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="H115" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I115" s="6" t="n"/>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="H121" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I121" s="6" t="n"/>
@@ -6222,7 +6222,7 @@
       </c>
       <c r="H158" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I158" s="6" t="n"/>
@@ -6749,7 +6749,7 @@
       </c>
       <c r="H173" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I173" s="6" t="n"/>
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H174" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I174" s="6" t="n"/>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="H175" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I175" s="6" t="n"/>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="H188" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I188" s="6" t="n"/>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H189" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I189" s="6" t="n"/>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="H192" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I192" s="6" t="n"/>
@@ -7501,7 +7501,7 @@
       </c>
       <c r="H193" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I193" s="6" t="n"/>
@@ -7694,7 +7694,7 @@
       </c>
       <c r="H198" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I198" s="6" t="n"/>
@@ -7735,7 +7735,7 @@
       </c>
       <c r="H199" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I199" s="6" t="n"/>
@@ -7776,7 +7776,7 @@
       </c>
       <c r="H200" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I200" s="6" t="n"/>
@@ -7854,7 +7854,7 @@
       </c>
       <c r="H202" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I202" s="6" t="n"/>
@@ -7895,7 +7895,7 @@
       </c>
       <c r="H203" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I203" s="6" t="n"/>
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H218" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I218" s="6" t="n"/>
@@ -9091,7 +9091,7 @@
       </c>
       <c r="H235" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I235" s="6" t="n"/>
@@ -9210,7 +9210,7 @@
       </c>
       <c r="H238" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I238" s="6" t="n"/>
@@ -9251,7 +9251,7 @@
       </c>
       <c r="H239" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I239" s="6" t="n"/>
@@ -9473,7 +9473,7 @@
       </c>
       <c r="H245" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I245" s="6" t="n"/>
@@ -10757,7 +10757,7 @@
       </c>
       <c r="H281" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I281" s="6" t="n"/>
@@ -10798,7 +10798,7 @@
       </c>
       <c r="H282" s="15" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I282" s="6" t="n"/>
@@ -10839,7 +10839,7 @@
       </c>
       <c r="H283" s="9" t="inlineStr">
         <is>
-          <t>Liste IFDC 2026</t>
+          <t>Liste du fournisseur</t>
         </is>
       </c>
       <c r="I283" s="6" t="n"/>
@@ -11233,7 +11233,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Source du prix — « Liste IFDC 2026 » si le prix vient du fichier de prix fourni,</t>
+          <t>Source du prix — « Liste supplier 2026 » si le prix vient du fichier de prix fourni,</t>
         </is>
       </c>
     </row>

</xml_diff>